<commit_message>
The start of lab 8
</commit_message>
<xml_diff>
--- a/Lab 5/Lab5-Forces and Vectors.xlsx
+++ b/Lab 5/Lab5-Forces and Vectors.xlsx
@@ -5,10 +5,10 @@
   <workbookPr date1904="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ngocb\Downloads\Book\Course\Physic Lab\Lab Assignment\Week 5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ngocb\Downloads\Book\Course\Physic Lab\Lab Assignment\Lab 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{583D5DCF-0841-4D0C-95E4-36676731EC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3727E0AE-3CA0-4926-9920-8DAD121ABCFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,15 +32,12 @@
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="16">
   <si>
     <t>Force</t>
   </si>
@@ -83,6 +80,12 @@
   <si>
     <t>30 DEGREE</t>
   </si>
+  <si>
+    <t>force</t>
+  </si>
+  <si>
+    <t>Magnitude (N)</t>
+  </si>
 </sst>
 </file>
 
@@ -92,7 +95,7 @@
     <numFmt numFmtId="164" formatCode=".00"/>
     <numFmt numFmtId="165" formatCode=".0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Geneva"/>
@@ -117,8 +120,42 @@
       <sz val="14"/>
       <name val="Geneva"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -131,8 +168,26 @@
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -175,11 +230,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -202,17 +309,12 @@
     <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -246,7 +348,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -278,6 +388,62 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,7 +595,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>234.92315519647701</c:v>
+                  <c:v>2.2999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -444,7 +610,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-85.505035831417359</c:v>
+                  <c:v>-0.84</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -718,7 +884,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-99.93775716230374</c:v>
+                  <c:v>-0.98</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -733,7 +899,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-75.36429722356803</c:v>
+                  <c:v>-0.74</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1007,7 +1173,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-134.98539803417327</c:v>
+                  <c:v>-1.32</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1022,7 +1188,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>160.86933305498539</c:v>
+                  <c:v>1.58</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1103,7 +1269,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-134.98539803417327</c:v>
+                  <c:v>-1.32</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1118,7 +1284,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>160.86933305498539</c:v>
+                  <c:v>1.58</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1392,7 +1558,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-99.93775716230374</c:v>
+                  <c:v>-0.98</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1407,7 +1573,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-75.36429722356803</c:v>
+                  <c:v>-0.74</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1493,7 +1659,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-134.98539803417327</c:v>
+                  <c:v>-1.32</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1508,7 +1674,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>160.86933305498539</c:v>
+                  <c:v>1.58</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1594,7 +1760,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>234.92315519647701</c:v>
+                  <c:v>2.2999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1609,7 +1775,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-85.505035831417359</c:v>
+                  <c:v>-0.84</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1870,7 +2036,7 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>4852</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>19080</xdr:rowOff>
+      <xdr:rowOff>19081</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2161,30 +2327,42 @@
     <col min="7" max="257" width="21.109375" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:257" ht="17.399999999999999">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:257" ht="18.600000000000001" thickBot="1">
+      <c r="A1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="38" t="s">
+      <c r="B1" s="67" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="67" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="39" t="s">
+        <v>2</v>
+      </c>
+      <c r="L1" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" s="37" t="s">
+        <v>4</v>
+      </c>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
@@ -2430,906 +2608,964 @@
       <c r="IV1" s="1"/>
       <c r="IW1" s="1"/>
     </row>
-    <row r="2" spans="1:257" ht="17.399999999999999">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:257" ht="18.600000000000001" thickBot="1">
+      <c r="A2" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="9">
-        <v>210</v>
-      </c>
-      <c r="C2" s="9">
+      <c r="B2" s="69">
+        <v>2.0579999999999998</v>
+      </c>
+      <c r="C2" s="69">
         <v>130</v>
       </c>
-      <c r="D2" s="39">
-        <f>B2*COS(C2/180*PI())</f>
+      <c r="D2" s="70">
+        <v>-1.32</v>
+      </c>
+      <c r="E2" s="70">
+        <v>1.58</v>
+      </c>
+      <c r="F2" s="10"/>
+      <c r="G2" s="35">
+        <v>30</v>
+      </c>
+      <c r="H2" s="10">
+        <f>(G2/1000)*9.8</f>
+        <v>0.29399999999999998</v>
+      </c>
+      <c r="I2" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="63">
+        <v>150</v>
+      </c>
+      <c r="K2" s="63">
+        <v>0</v>
+      </c>
+      <c r="L2" s="40">
         <v>-134.98539803417327</v>
       </c>
-      <c r="E2" s="39">
-        <f>B2*SIN(C2/180*PI())</f>
+      <c r="M2" s="40">
         <v>160.86933305498539</v>
       </c>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11">
-        <v>130</v>
-      </c>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="11"/>
-      <c r="T2" s="11"/>
-      <c r="U2" s="11"/>
-      <c r="V2" s="11"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="11"/>
-      <c r="Z2" s="11"/>
-      <c r="AA2" s="11"/>
-      <c r="AB2" s="11"/>
-      <c r="AC2" s="11"/>
-      <c r="AD2" s="11"/>
-      <c r="AE2" s="11"/>
-      <c r="AF2" s="11"/>
-      <c r="AG2" s="11"/>
-      <c r="AH2" s="11"/>
-      <c r="AI2" s="11"/>
-      <c r="AJ2" s="11"/>
-      <c r="AK2" s="11"/>
-      <c r="AL2" s="11"/>
-      <c r="AM2" s="11"/>
-      <c r="AN2" s="11"/>
-      <c r="AO2" s="11"/>
-      <c r="AP2" s="11"/>
-      <c r="AQ2" s="11"/>
-      <c r="AR2" s="11"/>
-      <c r="AS2" s="11"/>
-      <c r="AT2" s="11"/>
-      <c r="AU2" s="11"/>
-      <c r="AV2" s="11"/>
-      <c r="AW2" s="11"/>
-      <c r="AX2" s="11"/>
-      <c r="AY2" s="11"/>
-      <c r="AZ2" s="11"/>
-      <c r="BA2" s="11"/>
-      <c r="BB2" s="11"/>
-      <c r="BC2" s="11"/>
-      <c r="BD2" s="11"/>
-      <c r="BE2" s="11"/>
-      <c r="BF2" s="11"/>
-      <c r="BG2" s="11"/>
-      <c r="BH2" s="11"/>
-      <c r="BI2" s="11"/>
-      <c r="BJ2" s="11"/>
-      <c r="BK2" s="11"/>
-      <c r="BL2" s="11"/>
-      <c r="BM2" s="11"/>
-      <c r="BN2" s="11"/>
-      <c r="BO2" s="11"/>
-      <c r="BP2" s="11"/>
-      <c r="BQ2" s="11"/>
-      <c r="BR2" s="11"/>
-      <c r="BS2" s="11"/>
-      <c r="BT2" s="11"/>
-      <c r="BU2" s="11"/>
-      <c r="BV2" s="11"/>
-      <c r="BW2" s="11"/>
-      <c r="BX2" s="11"/>
-      <c r="BY2" s="11"/>
-      <c r="BZ2" s="11"/>
-      <c r="CA2" s="11"/>
-      <c r="CB2" s="11"/>
-      <c r="CC2" s="11"/>
-      <c r="CD2" s="11"/>
-      <c r="CE2" s="11"/>
-      <c r="CF2" s="11"/>
-      <c r="CG2" s="11"/>
-      <c r="CH2" s="11"/>
-      <c r="CI2" s="11"/>
-      <c r="CJ2" s="11"/>
-      <c r="CK2" s="11"/>
-      <c r="CL2" s="11"/>
-      <c r="CM2" s="11"/>
-      <c r="CN2" s="11"/>
-      <c r="CO2" s="11"/>
-      <c r="CP2" s="11"/>
-      <c r="CQ2" s="11"/>
-      <c r="CR2" s="11"/>
-      <c r="CS2" s="11"/>
-      <c r="CT2" s="11"/>
-      <c r="CU2" s="11"/>
-      <c r="CV2" s="11"/>
-      <c r="CW2" s="11"/>
-      <c r="CX2" s="11"/>
-      <c r="CY2" s="11"/>
-      <c r="CZ2" s="11"/>
-      <c r="DA2" s="11"/>
-      <c r="DB2" s="11"/>
-      <c r="DC2" s="11"/>
-      <c r="DD2" s="11"/>
-      <c r="DE2" s="11"/>
-      <c r="DF2" s="11"/>
-      <c r="DG2" s="11"/>
-      <c r="DH2" s="11"/>
-      <c r="DI2" s="11"/>
-      <c r="DJ2" s="11"/>
-      <c r="DK2" s="11"/>
-      <c r="DL2" s="11"/>
-      <c r="DM2" s="11"/>
-      <c r="DN2" s="11"/>
-      <c r="DO2" s="11"/>
-      <c r="DP2" s="11"/>
-      <c r="DQ2" s="11"/>
-      <c r="DR2" s="11"/>
-      <c r="DS2" s="11"/>
-      <c r="DT2" s="11"/>
-      <c r="DU2" s="11"/>
-      <c r="DV2" s="11"/>
-      <c r="DW2" s="11"/>
-      <c r="DX2" s="11"/>
-      <c r="DY2" s="11"/>
-      <c r="DZ2" s="11"/>
-      <c r="EA2" s="11"/>
-      <c r="EB2" s="11"/>
-      <c r="EC2" s="11"/>
-      <c r="ED2" s="11"/>
-      <c r="EE2" s="11"/>
-      <c r="EF2" s="11"/>
-      <c r="EG2" s="11"/>
-      <c r="EH2" s="11"/>
-      <c r="EI2" s="11"/>
-      <c r="EJ2" s="11"/>
-      <c r="EK2" s="11"/>
-      <c r="EL2" s="11"/>
-      <c r="EM2" s="11"/>
-      <c r="EN2" s="11"/>
-      <c r="EO2" s="11"/>
-      <c r="EP2" s="11"/>
-      <c r="EQ2" s="11"/>
-      <c r="ER2" s="11"/>
-      <c r="ES2" s="11"/>
-      <c r="ET2" s="11"/>
-      <c r="EU2" s="11"/>
-      <c r="EV2" s="11"/>
-      <c r="EW2" s="11"/>
-      <c r="EX2" s="11"/>
-      <c r="EY2" s="11"/>
-      <c r="EZ2" s="11"/>
-      <c r="FA2" s="11"/>
-      <c r="FB2" s="11"/>
-      <c r="FC2" s="11"/>
-      <c r="FD2" s="11"/>
-      <c r="FE2" s="11"/>
-      <c r="FF2" s="11"/>
-      <c r="FG2" s="11"/>
-      <c r="FH2" s="11"/>
-      <c r="FI2" s="11"/>
-      <c r="FJ2" s="11"/>
-      <c r="FK2" s="11"/>
-      <c r="FL2" s="11"/>
-      <c r="FM2" s="11"/>
-      <c r="FN2" s="11"/>
-      <c r="FO2" s="11"/>
-      <c r="FP2" s="11"/>
-      <c r="FQ2" s="11"/>
-      <c r="FR2" s="11"/>
-      <c r="FS2" s="11"/>
-      <c r="FT2" s="11"/>
-      <c r="FU2" s="11"/>
-      <c r="FV2" s="11"/>
-      <c r="FW2" s="11"/>
-      <c r="FX2" s="11"/>
-      <c r="FY2" s="11"/>
-      <c r="FZ2" s="11"/>
-      <c r="GA2" s="11"/>
-      <c r="GB2" s="11"/>
-      <c r="GC2" s="11"/>
-      <c r="GD2" s="11"/>
-      <c r="GE2" s="11"/>
-      <c r="GF2" s="11"/>
-      <c r="GG2" s="11"/>
-      <c r="GH2" s="11"/>
-      <c r="GI2" s="11"/>
-      <c r="GJ2" s="11"/>
-      <c r="GK2" s="11"/>
-      <c r="GL2" s="11"/>
-      <c r="GM2" s="11"/>
-      <c r="GN2" s="11"/>
-      <c r="GO2" s="11"/>
-      <c r="GP2" s="11"/>
-      <c r="GQ2" s="11"/>
-      <c r="GR2" s="11"/>
-      <c r="GS2" s="11"/>
-      <c r="GT2" s="11"/>
-      <c r="GU2" s="11"/>
-      <c r="GV2" s="11"/>
-      <c r="GW2" s="11"/>
-      <c r="GX2" s="11"/>
-      <c r="GY2" s="11"/>
-      <c r="GZ2" s="11"/>
-      <c r="HA2" s="11"/>
-      <c r="HB2" s="11"/>
-      <c r="HC2" s="11"/>
-      <c r="HD2" s="11"/>
-      <c r="HE2" s="11"/>
-      <c r="HF2" s="11"/>
-      <c r="HG2" s="11"/>
-      <c r="HH2" s="11"/>
-      <c r="HI2" s="11"/>
-      <c r="HJ2" s="11"/>
-      <c r="HK2" s="11"/>
-      <c r="HL2" s="11"/>
-      <c r="HM2" s="11"/>
-      <c r="HN2" s="11"/>
-      <c r="HO2" s="11"/>
-      <c r="HP2" s="11"/>
-      <c r="HQ2" s="11"/>
-      <c r="HR2" s="11"/>
-      <c r="HS2" s="11"/>
-      <c r="HT2" s="11"/>
-      <c r="HU2" s="11"/>
-      <c r="HV2" s="11"/>
-      <c r="HW2" s="11"/>
-      <c r="HX2" s="11"/>
-      <c r="HY2" s="11"/>
-      <c r="HZ2" s="11"/>
-      <c r="IA2" s="11"/>
-      <c r="IB2" s="11"/>
-      <c r="IC2" s="11"/>
-      <c r="ID2" s="11"/>
-      <c r="IE2" s="11"/>
-      <c r="IF2" s="11"/>
-      <c r="IG2" s="11"/>
-      <c r="IH2" s="11"/>
-      <c r="II2" s="11"/>
-      <c r="IJ2" s="11"/>
-      <c r="IK2" s="11"/>
-      <c r="IL2" s="11"/>
-      <c r="IM2" s="11"/>
-      <c r="IN2" s="11"/>
-      <c r="IO2" s="11"/>
-      <c r="IP2" s="11"/>
-      <c r="IQ2" s="11"/>
-      <c r="IR2" s="11"/>
-      <c r="IS2" s="11"/>
-      <c r="IT2" s="11"/>
-      <c r="IU2" s="11"/>
-      <c r="IV2" s="11"/>
-      <c r="IW2" s="11"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
+      <c r="AA2" s="10"/>
+      <c r="AB2" s="10"/>
+      <c r="AC2" s="10"/>
+      <c r="AD2" s="10"/>
+      <c r="AE2" s="10"/>
+      <c r="AF2" s="10"/>
+      <c r="AG2" s="10"/>
+      <c r="AH2" s="10"/>
+      <c r="AI2" s="10"/>
+      <c r="AJ2" s="10"/>
+      <c r="AK2" s="10"/>
+      <c r="AL2" s="10"/>
+      <c r="AM2" s="10"/>
+      <c r="AN2" s="10"/>
+      <c r="AO2" s="10"/>
+      <c r="AP2" s="10"/>
+      <c r="AQ2" s="10"/>
+      <c r="AR2" s="10"/>
+      <c r="AS2" s="10"/>
+      <c r="AT2" s="10"/>
+      <c r="AU2" s="10"/>
+      <c r="AV2" s="10"/>
+      <c r="AW2" s="10"/>
+      <c r="AX2" s="10"/>
+      <c r="AY2" s="10"/>
+      <c r="AZ2" s="10"/>
+      <c r="BA2" s="10"/>
+      <c r="BB2" s="10"/>
+      <c r="BC2" s="10"/>
+      <c r="BD2" s="10"/>
+      <c r="BE2" s="10"/>
+      <c r="BF2" s="10"/>
+      <c r="BG2" s="10"/>
+      <c r="BH2" s="10"/>
+      <c r="BI2" s="10"/>
+      <c r="BJ2" s="10"/>
+      <c r="BK2" s="10"/>
+      <c r="BL2" s="10"/>
+      <c r="BM2" s="10"/>
+      <c r="BN2" s="10"/>
+      <c r="BO2" s="10"/>
+      <c r="BP2" s="10"/>
+      <c r="BQ2" s="10"/>
+      <c r="BR2" s="10"/>
+      <c r="BS2" s="10"/>
+      <c r="BT2" s="10"/>
+      <c r="BU2" s="10"/>
+      <c r="BV2" s="10"/>
+      <c r="BW2" s="10"/>
+      <c r="BX2" s="10"/>
+      <c r="BY2" s="10"/>
+      <c r="BZ2" s="10"/>
+      <c r="CA2" s="10"/>
+      <c r="CB2" s="10"/>
+      <c r="CC2" s="10"/>
+      <c r="CD2" s="10"/>
+      <c r="CE2" s="10"/>
+      <c r="CF2" s="10"/>
+      <c r="CG2" s="10"/>
+      <c r="CH2" s="10"/>
+      <c r="CI2" s="10"/>
+      <c r="CJ2" s="10"/>
+      <c r="CK2" s="10"/>
+      <c r="CL2" s="10"/>
+      <c r="CM2" s="10"/>
+      <c r="CN2" s="10"/>
+      <c r="CO2" s="10"/>
+      <c r="CP2" s="10"/>
+      <c r="CQ2" s="10"/>
+      <c r="CR2" s="10"/>
+      <c r="CS2" s="10"/>
+      <c r="CT2" s="10"/>
+      <c r="CU2" s="10"/>
+      <c r="CV2" s="10"/>
+      <c r="CW2" s="10"/>
+      <c r="CX2" s="10"/>
+      <c r="CY2" s="10"/>
+      <c r="CZ2" s="10"/>
+      <c r="DA2" s="10"/>
+      <c r="DB2" s="10"/>
+      <c r="DC2" s="10"/>
+      <c r="DD2" s="10"/>
+      <c r="DE2" s="10"/>
+      <c r="DF2" s="10"/>
+      <c r="DG2" s="10"/>
+      <c r="DH2" s="10"/>
+      <c r="DI2" s="10"/>
+      <c r="DJ2" s="10"/>
+      <c r="DK2" s="10"/>
+      <c r="DL2" s="10"/>
+      <c r="DM2" s="10"/>
+      <c r="DN2" s="10"/>
+      <c r="DO2" s="10"/>
+      <c r="DP2" s="10"/>
+      <c r="DQ2" s="10"/>
+      <c r="DR2" s="10"/>
+      <c r="DS2" s="10"/>
+      <c r="DT2" s="10"/>
+      <c r="DU2" s="10"/>
+      <c r="DV2" s="10"/>
+      <c r="DW2" s="10"/>
+      <c r="DX2" s="10"/>
+      <c r="DY2" s="10"/>
+      <c r="DZ2" s="10"/>
+      <c r="EA2" s="10"/>
+      <c r="EB2" s="10"/>
+      <c r="EC2" s="10"/>
+      <c r="ED2" s="10"/>
+      <c r="EE2" s="10"/>
+      <c r="EF2" s="10"/>
+      <c r="EG2" s="10"/>
+      <c r="EH2" s="10"/>
+      <c r="EI2" s="10"/>
+      <c r="EJ2" s="10"/>
+      <c r="EK2" s="10"/>
+      <c r="EL2" s="10"/>
+      <c r="EM2" s="10"/>
+      <c r="EN2" s="10"/>
+      <c r="EO2" s="10"/>
+      <c r="EP2" s="10"/>
+      <c r="EQ2" s="10"/>
+      <c r="ER2" s="10"/>
+      <c r="ES2" s="10"/>
+      <c r="ET2" s="10"/>
+      <c r="EU2" s="10"/>
+      <c r="EV2" s="10"/>
+      <c r="EW2" s="10"/>
+      <c r="EX2" s="10"/>
+      <c r="EY2" s="10"/>
+      <c r="EZ2" s="10"/>
+      <c r="FA2" s="10"/>
+      <c r="FB2" s="10"/>
+      <c r="FC2" s="10"/>
+      <c r="FD2" s="10"/>
+      <c r="FE2" s="10"/>
+      <c r="FF2" s="10"/>
+      <c r="FG2" s="10"/>
+      <c r="FH2" s="10"/>
+      <c r="FI2" s="10"/>
+      <c r="FJ2" s="10"/>
+      <c r="FK2" s="10"/>
+      <c r="FL2" s="10"/>
+      <c r="FM2" s="10"/>
+      <c r="FN2" s="10"/>
+      <c r="FO2" s="10"/>
+      <c r="FP2" s="10"/>
+      <c r="FQ2" s="10"/>
+      <c r="FR2" s="10"/>
+      <c r="FS2" s="10"/>
+      <c r="FT2" s="10"/>
+      <c r="FU2" s="10"/>
+      <c r="FV2" s="10"/>
+      <c r="FW2" s="10"/>
+      <c r="FX2" s="10"/>
+      <c r="FY2" s="10"/>
+      <c r="FZ2" s="10"/>
+      <c r="GA2" s="10"/>
+      <c r="GB2" s="10"/>
+      <c r="GC2" s="10"/>
+      <c r="GD2" s="10"/>
+      <c r="GE2" s="10"/>
+      <c r="GF2" s="10"/>
+      <c r="GG2" s="10"/>
+      <c r="GH2" s="10"/>
+      <c r="GI2" s="10"/>
+      <c r="GJ2" s="10"/>
+      <c r="GK2" s="10"/>
+      <c r="GL2" s="10"/>
+      <c r="GM2" s="10"/>
+      <c r="GN2" s="10"/>
+      <c r="GO2" s="10"/>
+      <c r="GP2" s="10"/>
+      <c r="GQ2" s="10"/>
+      <c r="GR2" s="10"/>
+      <c r="GS2" s="10"/>
+      <c r="GT2" s="10"/>
+      <c r="GU2" s="10"/>
+      <c r="GV2" s="10"/>
+      <c r="GW2" s="10"/>
+      <c r="GX2" s="10"/>
+      <c r="GY2" s="10"/>
+      <c r="GZ2" s="10"/>
+      <c r="HA2" s="10"/>
+      <c r="HB2" s="10"/>
+      <c r="HC2" s="10"/>
+      <c r="HD2" s="10"/>
+      <c r="HE2" s="10"/>
+      <c r="HF2" s="10"/>
+      <c r="HG2" s="10"/>
+      <c r="HH2" s="10"/>
+      <c r="HI2" s="10"/>
+      <c r="HJ2" s="10"/>
+      <c r="HK2" s="10"/>
+      <c r="HL2" s="10"/>
+      <c r="HM2" s="10"/>
+      <c r="HN2" s="10"/>
+      <c r="HO2" s="10"/>
+      <c r="HP2" s="10"/>
+      <c r="HQ2" s="10"/>
+      <c r="HR2" s="10"/>
+      <c r="HS2" s="10"/>
+      <c r="HT2" s="10"/>
+      <c r="HU2" s="10"/>
+      <c r="HV2" s="10"/>
+      <c r="HW2" s="10"/>
+      <c r="HX2" s="10"/>
+      <c r="HY2" s="10"/>
+      <c r="HZ2" s="10"/>
+      <c r="IA2" s="10"/>
+      <c r="IB2" s="10"/>
+      <c r="IC2" s="10"/>
+      <c r="ID2" s="10"/>
+      <c r="IE2" s="10"/>
+      <c r="IF2" s="10"/>
+      <c r="IG2" s="10"/>
+      <c r="IH2" s="10"/>
+      <c r="II2" s="10"/>
+      <c r="IJ2" s="10"/>
+      <c r="IK2" s="10"/>
+      <c r="IL2" s="10"/>
+      <c r="IM2" s="10"/>
+      <c r="IN2" s="10"/>
+      <c r="IO2" s="10"/>
+      <c r="IP2" s="10"/>
+      <c r="IQ2" s="10"/>
+      <c r="IR2" s="10"/>
+      <c r="IS2" s="10"/>
+      <c r="IT2" s="10"/>
+      <c r="IU2" s="10"/>
+      <c r="IV2" s="10"/>
+      <c r="IW2" s="10"/>
     </row>
-    <row r="3" spans="1:257" ht="17.399999999999999">
-      <c r="A3" s="8" t="s">
+    <row r="3" spans="1:257" ht="18.600000000000001" thickBot="1">
+      <c r="A3" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="9">
-        <v>250</v>
-      </c>
-      <c r="C3" s="9">
+      <c r="B3" s="69">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="C3" s="69">
         <v>340</v>
       </c>
-      <c r="D3" s="39">
-        <f>B3*COS(C3/180*PI())</f>
+      <c r="D3" s="70">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E3" s="70">
+        <v>-0.84</v>
+      </c>
+      <c r="F3" s="10"/>
+      <c r="G3" s="33">
+        <v>4</v>
+      </c>
+      <c r="I3" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="63">
+        <v>200</v>
+      </c>
+      <c r="K3" s="63">
+        <v>90</v>
+      </c>
+      <c r="L3" s="40">
         <v>234.92315519647701</v>
       </c>
-      <c r="E3" s="39">
-        <f>B3*SIN(C3/180*PI())</f>
+      <c r="M3" s="40">
         <v>-85.505035831417359</v>
       </c>
-      <c r="F3" s="11">
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
+      <c r="Y3" s="10"/>
+      <c r="Z3" s="10"/>
+      <c r="AA3" s="10"/>
+      <c r="AB3" s="10"/>
+      <c r="AC3" s="10"/>
+      <c r="AD3" s="10"/>
+      <c r="AE3" s="10"/>
+      <c r="AF3" s="10"/>
+      <c r="AG3" s="10"/>
+      <c r="AH3" s="10"/>
+      <c r="AI3" s="10"/>
+      <c r="AJ3" s="10"/>
+      <c r="AK3" s="10"/>
+      <c r="AL3" s="10"/>
+      <c r="AM3" s="10"/>
+      <c r="AN3" s="10"/>
+      <c r="AO3" s="10"/>
+      <c r="AP3" s="10"/>
+      <c r="AQ3" s="10"/>
+      <c r="AR3" s="10"/>
+      <c r="AS3" s="10"/>
+      <c r="AT3" s="10"/>
+      <c r="AU3" s="10"/>
+      <c r="AV3" s="10"/>
+      <c r="AW3" s="10"/>
+      <c r="AX3" s="10"/>
+      <c r="AY3" s="10"/>
+      <c r="AZ3" s="10"/>
+      <c r="BA3" s="10"/>
+      <c r="BB3" s="10"/>
+      <c r="BC3" s="10"/>
+      <c r="BD3" s="10"/>
+      <c r="BE3" s="10"/>
+      <c r="BF3" s="10"/>
+      <c r="BG3" s="10"/>
+      <c r="BH3" s="10"/>
+      <c r="BI3" s="10"/>
+      <c r="BJ3" s="10"/>
+      <c r="BK3" s="10"/>
+      <c r="BL3" s="10"/>
+      <c r="BM3" s="10"/>
+      <c r="BN3" s="10"/>
+      <c r="BO3" s="10"/>
+      <c r="BP3" s="10"/>
+      <c r="BQ3" s="10"/>
+      <c r="BR3" s="10"/>
+      <c r="BS3" s="10"/>
+      <c r="BT3" s="10"/>
+      <c r="BU3" s="10"/>
+      <c r="BV3" s="10"/>
+      <c r="BW3" s="10"/>
+      <c r="BX3" s="10"/>
+      <c r="BY3" s="10"/>
+      <c r="BZ3" s="10"/>
+      <c r="CA3" s="10"/>
+      <c r="CB3" s="10"/>
+      <c r="CC3" s="10"/>
+      <c r="CD3" s="10"/>
+      <c r="CE3" s="10"/>
+      <c r="CF3" s="10"/>
+      <c r="CG3" s="10"/>
+      <c r="CH3" s="10"/>
+      <c r="CI3" s="10"/>
+      <c r="CJ3" s="10"/>
+      <c r="CK3" s="10"/>
+      <c r="CL3" s="10"/>
+      <c r="CM3" s="10"/>
+      <c r="CN3" s="10"/>
+      <c r="CO3" s="10"/>
+      <c r="CP3" s="10"/>
+      <c r="CQ3" s="10"/>
+      <c r="CR3" s="10"/>
+      <c r="CS3" s="10"/>
+      <c r="CT3" s="10"/>
+      <c r="CU3" s="10"/>
+      <c r="CV3" s="10"/>
+      <c r="CW3" s="10"/>
+      <c r="CX3" s="10"/>
+      <c r="CY3" s="10"/>
+      <c r="CZ3" s="10"/>
+      <c r="DA3" s="10"/>
+      <c r="DB3" s="10"/>
+      <c r="DC3" s="10"/>
+      <c r="DD3" s="10"/>
+      <c r="DE3" s="10"/>
+      <c r="DF3" s="10"/>
+      <c r="DG3" s="10"/>
+      <c r="DH3" s="10"/>
+      <c r="DI3" s="10"/>
+      <c r="DJ3" s="10"/>
+      <c r="DK3" s="10"/>
+      <c r="DL3" s="10"/>
+      <c r="DM3" s="10"/>
+      <c r="DN3" s="10"/>
+      <c r="DO3" s="10"/>
+      <c r="DP3" s="10"/>
+      <c r="DQ3" s="10"/>
+      <c r="DR3" s="10"/>
+      <c r="DS3" s="10"/>
+      <c r="DT3" s="10"/>
+      <c r="DU3" s="10"/>
+      <c r="DV3" s="10"/>
+      <c r="DW3" s="10"/>
+      <c r="DX3" s="10"/>
+      <c r="DY3" s="10"/>
+      <c r="DZ3" s="10"/>
+      <c r="EA3" s="10"/>
+      <c r="EB3" s="10"/>
+      <c r="EC3" s="10"/>
+      <c r="ED3" s="10"/>
+      <c r="EE3" s="10"/>
+      <c r="EF3" s="10"/>
+      <c r="EG3" s="10"/>
+      <c r="EH3" s="10"/>
+      <c r="EI3" s="10"/>
+      <c r="EJ3" s="10"/>
+      <c r="EK3" s="10"/>
+      <c r="EL3" s="10"/>
+      <c r="EM3" s="10"/>
+      <c r="EN3" s="10"/>
+      <c r="EO3" s="10"/>
+      <c r="EP3" s="10"/>
+      <c r="EQ3" s="10"/>
+      <c r="ER3" s="10"/>
+      <c r="ES3" s="10"/>
+      <c r="ET3" s="10"/>
+      <c r="EU3" s="10"/>
+      <c r="EV3" s="10"/>
+      <c r="EW3" s="10"/>
+      <c r="EX3" s="10"/>
+      <c r="EY3" s="10"/>
+      <c r="EZ3" s="10"/>
+      <c r="FA3" s="10"/>
+      <c r="FB3" s="10"/>
+      <c r="FC3" s="10"/>
+      <c r="FD3" s="10"/>
+      <c r="FE3" s="10"/>
+      <c r="FF3" s="10"/>
+      <c r="FG3" s="10"/>
+      <c r="FH3" s="10"/>
+      <c r="FI3" s="10"/>
+      <c r="FJ3" s="10"/>
+      <c r="FK3" s="10"/>
+      <c r="FL3" s="10"/>
+      <c r="FM3" s="10"/>
+      <c r="FN3" s="10"/>
+      <c r="FO3" s="10"/>
+      <c r="FP3" s="10"/>
+      <c r="FQ3" s="10"/>
+      <c r="FR3" s="10"/>
+      <c r="FS3" s="10"/>
+      <c r="FT3" s="10"/>
+      <c r="FU3" s="10"/>
+      <c r="FV3" s="10"/>
+      <c r="FW3" s="10"/>
+      <c r="FX3" s="10"/>
+      <c r="FY3" s="10"/>
+      <c r="FZ3" s="10"/>
+      <c r="GA3" s="10"/>
+      <c r="GB3" s="10"/>
+      <c r="GC3" s="10"/>
+      <c r="GD3" s="10"/>
+      <c r="GE3" s="10"/>
+      <c r="GF3" s="10"/>
+      <c r="GG3" s="10"/>
+      <c r="GH3" s="10"/>
+      <c r="GI3" s="10"/>
+      <c r="GJ3" s="10"/>
+      <c r="GK3" s="10"/>
+      <c r="GL3" s="10"/>
+      <c r="GM3" s="10"/>
+      <c r="GN3" s="10"/>
+      <c r="GO3" s="10"/>
+      <c r="GP3" s="10"/>
+      <c r="GQ3" s="10"/>
+      <c r="GR3" s="10"/>
+      <c r="GS3" s="10"/>
+      <c r="GT3" s="10"/>
+      <c r="GU3" s="10"/>
+      <c r="GV3" s="10"/>
+      <c r="GW3" s="10"/>
+      <c r="GX3" s="10"/>
+      <c r="GY3" s="10"/>
+      <c r="GZ3" s="10"/>
+      <c r="HA3" s="10"/>
+      <c r="HB3" s="10"/>
+      <c r="HC3" s="10"/>
+      <c r="HD3" s="10"/>
+      <c r="HE3" s="10"/>
+      <c r="HF3" s="10"/>
+      <c r="HG3" s="10"/>
+      <c r="HH3" s="10"/>
+      <c r="HI3" s="10"/>
+      <c r="HJ3" s="10"/>
+      <c r="HK3" s="10"/>
+      <c r="HL3" s="10"/>
+      <c r="HM3" s="10"/>
+      <c r="HN3" s="10"/>
+      <c r="HO3" s="10"/>
+      <c r="HP3" s="10"/>
+      <c r="HQ3" s="10"/>
+      <c r="HR3" s="10"/>
+      <c r="HS3" s="10"/>
+      <c r="HT3" s="10"/>
+      <c r="HU3" s="10"/>
+      <c r="HV3" s="10"/>
+      <c r="HW3" s="10"/>
+      <c r="HX3" s="10"/>
+      <c r="HY3" s="10"/>
+      <c r="HZ3" s="10"/>
+      <c r="IA3" s="10"/>
+      <c r="IB3" s="10"/>
+      <c r="IC3" s="10"/>
+      <c r="ID3" s="10"/>
+      <c r="IE3" s="10"/>
+      <c r="IF3" s="10"/>
+      <c r="IG3" s="10"/>
+      <c r="IH3" s="10"/>
+      <c r="II3" s="10"/>
+      <c r="IJ3" s="10"/>
+      <c r="IK3" s="10"/>
+      <c r="IL3" s="10"/>
+      <c r="IM3" s="10"/>
+      <c r="IN3" s="10"/>
+      <c r="IO3" s="10"/>
+      <c r="IP3" s="10"/>
+      <c r="IQ3" s="10"/>
+      <c r="IR3" s="10"/>
+      <c r="IS3" s="10"/>
+      <c r="IT3" s="10"/>
+      <c r="IU3" s="10"/>
+      <c r="IV3" s="10"/>
+      <c r="IW3" s="10"/>
+    </row>
+    <row r="4" spans="1:257" ht="18.600000000000001" thickBot="1">
+      <c r="A4" s="68" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="69">
+        <v>1.2266999999999999</v>
+      </c>
+      <c r="C4" s="69">
+        <v>217.02</v>
+      </c>
+      <c r="D4" s="70">
+        <v>-0.98</v>
+      </c>
+      <c r="E4" s="70">
+        <v>-0.74</v>
+      </c>
+      <c r="I4" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="65">
+        <v>125.16921587448687</v>
+      </c>
+      <c r="K4" s="65">
+        <v>217.02039733055338</v>
+      </c>
+      <c r="L4" s="40">
+        <v>-99.93775716230374</v>
+      </c>
+      <c r="M4" s="40">
+        <v>-75.36429722356803</v>
+      </c>
+    </row>
+    <row r="5" spans="1:257" ht="18.600000000000001" thickBot="1">
+      <c r="A5" s="68" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="69">
+        <v>1.1956</v>
+      </c>
+      <c r="C5" s="69">
+        <v>215</v>
+      </c>
+      <c r="D5" s="71" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="72"/>
+      <c r="F5" s="31"/>
+      <c r="I5" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" s="64">
+        <v>122</v>
+      </c>
+      <c r="K5" s="63">
+        <v>215</v>
+      </c>
+      <c r="L5" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="M5" s="42"/>
+    </row>
+    <row r="6" spans="1:257" ht="18.600000000000001" thickBot="1">
+      <c r="A6" s="68" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="70">
+        <v>0.04</v>
+      </c>
+      <c r="C6" s="70">
+        <v>2.02</v>
+      </c>
+      <c r="D6" s="71" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="72"/>
+      <c r="F6" s="31"/>
+      <c r="I6" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="J6" s="40">
+        <v>3.1692158744868664</v>
+      </c>
+      <c r="K6" s="40">
+        <v>2.0203973305533793</v>
+      </c>
+      <c r="L6" s="43" t="s">
+        <v>9</v>
+      </c>
+      <c r="M6" s="42"/>
+    </row>
+    <row r="7" spans="1:257" ht="18.600000000000001" thickBot="1">
+      <c r="A7" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="70">
+        <v>3.03</v>
+      </c>
+      <c r="C7" s="71"/>
+      <c r="D7" s="71" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="72"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="10">
         <v>30</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="4">
-        <v>340</v>
-      </c>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
-      <c r="S3" s="11"/>
-      <c r="T3" s="11"/>
-      <c r="U3" s="11"/>
-      <c r="V3" s="11"/>
-      <c r="W3" s="11"/>
-      <c r="X3" s="11"/>
-      <c r="Y3" s="11"/>
-      <c r="Z3" s="11"/>
-      <c r="AA3" s="11"/>
-      <c r="AB3" s="11"/>
-      <c r="AC3" s="11"/>
-      <c r="AD3" s="11"/>
-      <c r="AE3" s="11"/>
-      <c r="AF3" s="11"/>
-      <c r="AG3" s="11"/>
-      <c r="AH3" s="11"/>
-      <c r="AI3" s="11"/>
-      <c r="AJ3" s="11"/>
-      <c r="AK3" s="11"/>
-      <c r="AL3" s="11"/>
-      <c r="AM3" s="11"/>
-      <c r="AN3" s="11"/>
-      <c r="AO3" s="11"/>
-      <c r="AP3" s="11"/>
-      <c r="AQ3" s="11"/>
-      <c r="AR3" s="11"/>
-      <c r="AS3" s="11"/>
-      <c r="AT3" s="11"/>
-      <c r="AU3" s="11"/>
-      <c r="AV3" s="11"/>
-      <c r="AW3" s="11"/>
-      <c r="AX3" s="11"/>
-      <c r="AY3" s="11"/>
-      <c r="AZ3" s="11"/>
-      <c r="BA3" s="11"/>
-      <c r="BB3" s="11"/>
-      <c r="BC3" s="11"/>
-      <c r="BD3" s="11"/>
-      <c r="BE3" s="11"/>
-      <c r="BF3" s="11"/>
-      <c r="BG3" s="11"/>
-      <c r="BH3" s="11"/>
-      <c r="BI3" s="11"/>
-      <c r="BJ3" s="11"/>
-      <c r="BK3" s="11"/>
-      <c r="BL3" s="11"/>
-      <c r="BM3" s="11"/>
-      <c r="BN3" s="11"/>
-      <c r="BO3" s="11"/>
-      <c r="BP3" s="11"/>
-      <c r="BQ3" s="11"/>
-      <c r="BR3" s="11"/>
-      <c r="BS3" s="11"/>
-      <c r="BT3" s="11"/>
-      <c r="BU3" s="11"/>
-      <c r="BV3" s="11"/>
-      <c r="BW3" s="11"/>
-      <c r="BX3" s="11"/>
-      <c r="BY3" s="11"/>
-      <c r="BZ3" s="11"/>
-      <c r="CA3" s="11"/>
-      <c r="CB3" s="11"/>
-      <c r="CC3" s="11"/>
-      <c r="CD3" s="11"/>
-      <c r="CE3" s="11"/>
-      <c r="CF3" s="11"/>
-      <c r="CG3" s="11"/>
-      <c r="CH3" s="11"/>
-      <c r="CI3" s="11"/>
-      <c r="CJ3" s="11"/>
-      <c r="CK3" s="11"/>
-      <c r="CL3" s="11"/>
-      <c r="CM3" s="11"/>
-      <c r="CN3" s="11"/>
-      <c r="CO3" s="11"/>
-      <c r="CP3" s="11"/>
-      <c r="CQ3" s="11"/>
-      <c r="CR3" s="11"/>
-      <c r="CS3" s="11"/>
-      <c r="CT3" s="11"/>
-      <c r="CU3" s="11"/>
-      <c r="CV3" s="11"/>
-      <c r="CW3" s="11"/>
-      <c r="CX3" s="11"/>
-      <c r="CY3" s="11"/>
-      <c r="CZ3" s="11"/>
-      <c r="DA3" s="11"/>
-      <c r="DB3" s="11"/>
-      <c r="DC3" s="11"/>
-      <c r="DD3" s="11"/>
-      <c r="DE3" s="11"/>
-      <c r="DF3" s="11"/>
-      <c r="DG3" s="11"/>
-      <c r="DH3" s="11"/>
-      <c r="DI3" s="11"/>
-      <c r="DJ3" s="11"/>
-      <c r="DK3" s="11"/>
-      <c r="DL3" s="11"/>
-      <c r="DM3" s="11"/>
-      <c r="DN3" s="11"/>
-      <c r="DO3" s="11"/>
-      <c r="DP3" s="11"/>
-      <c r="DQ3" s="11"/>
-      <c r="DR3" s="11"/>
-      <c r="DS3" s="11"/>
-      <c r="DT3" s="11"/>
-      <c r="DU3" s="11"/>
-      <c r="DV3" s="11"/>
-      <c r="DW3" s="11"/>
-      <c r="DX3" s="11"/>
-      <c r="DY3" s="11"/>
-      <c r="DZ3" s="11"/>
-      <c r="EA3" s="11"/>
-      <c r="EB3" s="11"/>
-      <c r="EC3" s="11"/>
-      <c r="ED3" s="11"/>
-      <c r="EE3" s="11"/>
-      <c r="EF3" s="11"/>
-      <c r="EG3" s="11"/>
-      <c r="EH3" s="11"/>
-      <c r="EI3" s="11"/>
-      <c r="EJ3" s="11"/>
-      <c r="EK3" s="11"/>
-      <c r="EL3" s="11"/>
-      <c r="EM3" s="11"/>
-      <c r="EN3" s="11"/>
-      <c r="EO3" s="11"/>
-      <c r="EP3" s="11"/>
-      <c r="EQ3" s="11"/>
-      <c r="ER3" s="11"/>
-      <c r="ES3" s="11"/>
-      <c r="ET3" s="11"/>
-      <c r="EU3" s="11"/>
-      <c r="EV3" s="11"/>
-      <c r="EW3" s="11"/>
-      <c r="EX3" s="11"/>
-      <c r="EY3" s="11"/>
-      <c r="EZ3" s="11"/>
-      <c r="FA3" s="11"/>
-      <c r="FB3" s="11"/>
-      <c r="FC3" s="11"/>
-      <c r="FD3" s="11"/>
-      <c r="FE3" s="11"/>
-      <c r="FF3" s="11"/>
-      <c r="FG3" s="11"/>
-      <c r="FH3" s="11"/>
-      <c r="FI3" s="11"/>
-      <c r="FJ3" s="11"/>
-      <c r="FK3" s="11"/>
-      <c r="FL3" s="11"/>
-      <c r="FM3" s="11"/>
-      <c r="FN3" s="11"/>
-      <c r="FO3" s="11"/>
-      <c r="FP3" s="11"/>
-      <c r="FQ3" s="11"/>
-      <c r="FR3" s="11"/>
-      <c r="FS3" s="11"/>
-      <c r="FT3" s="11"/>
-      <c r="FU3" s="11"/>
-      <c r="FV3" s="11"/>
-      <c r="FW3" s="11"/>
-      <c r="FX3" s="11"/>
-      <c r="FY3" s="11"/>
-      <c r="FZ3" s="11"/>
-      <c r="GA3" s="11"/>
-      <c r="GB3" s="11"/>
-      <c r="GC3" s="11"/>
-      <c r="GD3" s="11"/>
-      <c r="GE3" s="11"/>
-      <c r="GF3" s="11"/>
-      <c r="GG3" s="11"/>
-      <c r="GH3" s="11"/>
-      <c r="GI3" s="11"/>
-      <c r="GJ3" s="11"/>
-      <c r="GK3" s="11"/>
-      <c r="GL3" s="11"/>
-      <c r="GM3" s="11"/>
-      <c r="GN3" s="11"/>
-      <c r="GO3" s="11"/>
-      <c r="GP3" s="11"/>
-      <c r="GQ3" s="11"/>
-      <c r="GR3" s="11"/>
-      <c r="GS3" s="11"/>
-      <c r="GT3" s="11"/>
-      <c r="GU3" s="11"/>
-      <c r="GV3" s="11"/>
-      <c r="GW3" s="11"/>
-      <c r="GX3" s="11"/>
-      <c r="GY3" s="11"/>
-      <c r="GZ3" s="11"/>
-      <c r="HA3" s="11"/>
-      <c r="HB3" s="11"/>
-      <c r="HC3" s="11"/>
-      <c r="HD3" s="11"/>
-      <c r="HE3" s="11"/>
-      <c r="HF3" s="11"/>
-      <c r="HG3" s="11"/>
-      <c r="HH3" s="11"/>
-      <c r="HI3" s="11"/>
-      <c r="HJ3" s="11"/>
-      <c r="HK3" s="11"/>
-      <c r="HL3" s="11"/>
-      <c r="HM3" s="11"/>
-      <c r="HN3" s="11"/>
-      <c r="HO3" s="11"/>
-      <c r="HP3" s="11"/>
-      <c r="HQ3" s="11"/>
-      <c r="HR3" s="11"/>
-      <c r="HS3" s="11"/>
-      <c r="HT3" s="11"/>
-      <c r="HU3" s="11"/>
-      <c r="HV3" s="11"/>
-      <c r="HW3" s="11"/>
-      <c r="HX3" s="11"/>
-      <c r="HY3" s="11"/>
-      <c r="HZ3" s="11"/>
-      <c r="IA3" s="11"/>
-      <c r="IB3" s="11"/>
-      <c r="IC3" s="11"/>
-      <c r="ID3" s="11"/>
-      <c r="IE3" s="11"/>
-      <c r="IF3" s="11"/>
-      <c r="IG3" s="11"/>
-      <c r="IH3" s="11"/>
-      <c r="II3" s="11"/>
-      <c r="IJ3" s="11"/>
-      <c r="IK3" s="11"/>
-      <c r="IL3" s="11"/>
-      <c r="IM3" s="11"/>
-      <c r="IN3" s="11"/>
-      <c r="IO3" s="11"/>
-      <c r="IP3" s="11"/>
-      <c r="IQ3" s="11"/>
-      <c r="IR3" s="11"/>
-      <c r="IS3" s="11"/>
-      <c r="IT3" s="11"/>
-      <c r="IU3" s="11"/>
-      <c r="IV3" s="11"/>
-      <c r="IW3" s="11"/>
-    </row>
-    <row r="4" spans="1:257" ht="17.399999999999999">
-      <c r="A4" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="39">
-        <f>(D4^2+E4^2)^0.5</f>
-        <v>125.16921587448687</v>
-      </c>
-      <c r="C4" s="39">
-        <f>IF(D4&lt;0,(IF(E4&lt;0,ATAN(E4/D4)*(180/PI())+180,ATAN(E4/D4)*(180/PI())+180)),(IF(E4&lt;0,ATAN(E4/D4)*(180/PI())+360,ATAN(E4/D4)*(180/PI()))))</f>
-        <v>217.02039733055338</v>
-      </c>
-      <c r="D4" s="39">
-        <f>-D2-D3</f>
-        <v>-99.93775716230374</v>
-      </c>
-      <c r="E4" s="39">
-        <f>-E2-E3</f>
-        <v>-75.36429722356803</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:257" ht="17.399999999999999">
-      <c r="A5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="13">
-        <v>122</v>
-      </c>
-      <c r="C5" s="9">
-        <v>215</v>
-      </c>
-      <c r="D5" s="40" t="s">
+      <c r="H7" s="15"/>
+      <c r="I7" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="44">
+        <v>2.5644098625099025</v>
+      </c>
+      <c r="K7" s="46"/>
+      <c r="L7" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="41"/>
-      <c r="F5" s="35"/>
-    </row>
-    <row r="6" spans="1:257" ht="17.399999999999999">
-      <c r="A6" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="39">
-        <f>B4-B5</f>
-        <v>3.1692158744868664</v>
-      </c>
-      <c r="C6" s="39">
-        <f>C4-C5</f>
-        <v>2.0203973305533793</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="41"/>
-      <c r="F6" s="35"/>
-    </row>
-    <row r="7" spans="1:257" ht="17.399999999999999">
-      <c r="A7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="43">
-        <f>ABS((B5-B4)/((B5+B4)/2))*100</f>
-        <v>2.5644098625099025</v>
-      </c>
-      <c r="C7" s="45"/>
-      <c r="D7" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="44"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-      <c r="O7" s="18"/>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="18"/>
-      <c r="T7" s="18"/>
-      <c r="U7" s="18"/>
-      <c r="V7" s="18"/>
-      <c r="W7" s="18"/>
-      <c r="X7" s="18"/>
-      <c r="Y7" s="18"/>
-      <c r="Z7" s="18"/>
-      <c r="AA7" s="18"/>
-      <c r="AB7" s="18"/>
-      <c r="AC7" s="18"/>
-      <c r="AD7" s="18"/>
-      <c r="AE7" s="18"/>
-      <c r="AF7" s="18"/>
-      <c r="AG7" s="18"/>
-      <c r="AH7" s="18"/>
-      <c r="AI7" s="18"/>
-      <c r="AJ7" s="18"/>
-      <c r="AK7" s="18"/>
-      <c r="AL7" s="18"/>
-      <c r="AM7" s="18"/>
-      <c r="AN7" s="18"/>
-      <c r="AO7" s="18"/>
-      <c r="AP7" s="18"/>
-      <c r="AQ7" s="18"/>
-      <c r="AR7" s="18"/>
-      <c r="AS7" s="18"/>
-      <c r="AT7" s="18"/>
-      <c r="AU7" s="18"/>
-      <c r="AV7" s="18"/>
-      <c r="AW7" s="18"/>
-      <c r="AX7" s="18"/>
-      <c r="AY7" s="18"/>
-      <c r="AZ7" s="18"/>
-      <c r="BA7" s="18"/>
-      <c r="BB7" s="18"/>
-      <c r="BC7" s="18"/>
-      <c r="BD7" s="18"/>
-      <c r="BE7" s="18"/>
-      <c r="BF7" s="18"/>
-      <c r="BG7" s="18"/>
-      <c r="BH7" s="18"/>
-      <c r="BI7" s="18"/>
-      <c r="BJ7" s="18"/>
-      <c r="BK7" s="18"/>
-      <c r="BL7" s="18"/>
-      <c r="BM7" s="18"/>
-      <c r="BN7" s="18"/>
-      <c r="BO7" s="18"/>
-      <c r="BP7" s="18"/>
-      <c r="BQ7" s="18"/>
-      <c r="BR7" s="18"/>
-      <c r="BS7" s="18"/>
-      <c r="BT7" s="18"/>
-      <c r="BU7" s="18"/>
-      <c r="BV7" s="18"/>
-      <c r="BW7" s="18"/>
-      <c r="BX7" s="18"/>
-      <c r="BY7" s="18"/>
-      <c r="BZ7" s="18"/>
-      <c r="CA7" s="18"/>
-      <c r="CB7" s="18"/>
-      <c r="CC7" s="18"/>
-      <c r="CD7" s="18"/>
-      <c r="CE7" s="18"/>
-      <c r="CF7" s="18"/>
-      <c r="CG7" s="18"/>
-      <c r="CH7" s="18"/>
-      <c r="CI7" s="18"/>
-      <c r="CJ7" s="18"/>
-      <c r="CK7" s="18"/>
-      <c r="CL7" s="18"/>
-      <c r="CM7" s="18"/>
-      <c r="CN7" s="18"/>
-      <c r="CO7" s="18"/>
-      <c r="CP7" s="18"/>
-      <c r="CQ7" s="18"/>
-      <c r="CR7" s="18"/>
-      <c r="CS7" s="18"/>
-      <c r="CT7" s="18"/>
-      <c r="CU7" s="18"/>
-      <c r="CV7" s="18"/>
-      <c r="CW7" s="18"/>
-      <c r="CX7" s="18"/>
-      <c r="CY7" s="18"/>
-      <c r="CZ7" s="18"/>
-      <c r="DA7" s="18"/>
-      <c r="DB7" s="18"/>
-      <c r="DC7" s="18"/>
-      <c r="DD7" s="18"/>
-      <c r="DE7" s="18"/>
-      <c r="DF7" s="18"/>
-      <c r="DG7" s="18"/>
-      <c r="DH7" s="18"/>
-      <c r="DI7" s="18"/>
-      <c r="DJ7" s="18"/>
-      <c r="DK7" s="18"/>
-      <c r="DL7" s="18"/>
-      <c r="DM7" s="18"/>
-      <c r="DN7" s="18"/>
-      <c r="DO7" s="18"/>
-      <c r="DP7" s="18"/>
-      <c r="DQ7" s="18"/>
-      <c r="DR7" s="18"/>
-      <c r="DS7" s="18"/>
-      <c r="DT7" s="18"/>
-      <c r="DU7" s="18"/>
-      <c r="DV7" s="18"/>
-      <c r="DW7" s="18"/>
-      <c r="DX7" s="18"/>
-      <c r="DY7" s="18"/>
-      <c r="DZ7" s="18"/>
-      <c r="EA7" s="18"/>
-      <c r="EB7" s="18"/>
-      <c r="EC7" s="18"/>
-      <c r="ED7" s="18"/>
-      <c r="EE7" s="18"/>
-      <c r="EF7" s="18"/>
-      <c r="EG7" s="18"/>
-      <c r="EH7" s="18"/>
-      <c r="EI7" s="18"/>
-      <c r="EJ7" s="18"/>
-      <c r="EK7" s="18"/>
-      <c r="EL7" s="18"/>
-      <c r="EM7" s="18"/>
-      <c r="EN7" s="18"/>
-      <c r="EO7" s="18"/>
-      <c r="EP7" s="18"/>
-      <c r="EQ7" s="18"/>
-      <c r="ER7" s="18"/>
-      <c r="ES7" s="18"/>
-      <c r="ET7" s="18"/>
-      <c r="EU7" s="18"/>
-      <c r="EV7" s="18"/>
-      <c r="EW7" s="18"/>
-      <c r="EX7" s="18"/>
-      <c r="EY7" s="18"/>
-      <c r="EZ7" s="18"/>
-      <c r="FA7" s="18"/>
-      <c r="FB7" s="18"/>
-      <c r="FC7" s="18"/>
-      <c r="FD7" s="18"/>
-      <c r="FE7" s="18"/>
-      <c r="FF7" s="18"/>
-      <c r="FG7" s="18"/>
-      <c r="FH7" s="18"/>
-      <c r="FI7" s="18"/>
-      <c r="FJ7" s="18"/>
-      <c r="FK7" s="18"/>
-      <c r="FL7" s="18"/>
-      <c r="FM7" s="18"/>
-      <c r="FN7" s="18"/>
-      <c r="FO7" s="18"/>
-      <c r="FP7" s="18"/>
-      <c r="FQ7" s="18"/>
-      <c r="FR7" s="18"/>
-      <c r="FS7" s="18"/>
-      <c r="FT7" s="18"/>
-      <c r="FU7" s="18"/>
-      <c r="FV7" s="18"/>
-      <c r="FW7" s="18"/>
-      <c r="FX7" s="18"/>
-      <c r="FY7" s="18"/>
-      <c r="FZ7" s="18"/>
-      <c r="GA7" s="18"/>
-      <c r="GB7" s="18"/>
-      <c r="GC7" s="18"/>
-      <c r="GD7" s="18"/>
-      <c r="GE7" s="18"/>
-      <c r="GF7" s="18"/>
-      <c r="GG7" s="18"/>
-      <c r="GH7" s="18"/>
-      <c r="GI7" s="18"/>
-      <c r="GJ7" s="18"/>
-      <c r="GK7" s="18"/>
-      <c r="GL7" s="18"/>
-      <c r="GM7" s="18"/>
-      <c r="GN7" s="18"/>
-      <c r="GO7" s="18"/>
-      <c r="GP7" s="18"/>
-      <c r="GQ7" s="18"/>
-      <c r="GR7" s="18"/>
-      <c r="GS7" s="18"/>
-      <c r="GT7" s="18"/>
-      <c r="GU7" s="18"/>
-      <c r="GV7" s="18"/>
-      <c r="GW7" s="18"/>
-      <c r="GX7" s="18"/>
-      <c r="GY7" s="18"/>
-      <c r="GZ7" s="18"/>
-      <c r="HA7" s="18"/>
-      <c r="HB7" s="18"/>
-      <c r="HC7" s="18"/>
-      <c r="HD7" s="18"/>
-      <c r="HE7" s="18"/>
-      <c r="HF7" s="18"/>
-      <c r="HG7" s="18"/>
-      <c r="HH7" s="18"/>
-      <c r="HI7" s="18"/>
-      <c r="HJ7" s="18"/>
-      <c r="HK7" s="18"/>
-      <c r="HL7" s="18"/>
-      <c r="HM7" s="18"/>
-      <c r="HN7" s="18"/>
-      <c r="HO7" s="18"/>
-      <c r="HP7" s="18"/>
-      <c r="HQ7" s="18"/>
-      <c r="HR7" s="18"/>
-      <c r="HS7" s="18"/>
-      <c r="HT7" s="18"/>
-      <c r="HU7" s="18"/>
-      <c r="HV7" s="18"/>
-      <c r="HW7" s="18"/>
-      <c r="HX7" s="18"/>
-      <c r="HY7" s="18"/>
-      <c r="HZ7" s="18"/>
-      <c r="IA7" s="18"/>
-      <c r="IB7" s="18"/>
-      <c r="IC7" s="18"/>
-      <c r="ID7" s="18"/>
-      <c r="IE7" s="18"/>
-      <c r="IF7" s="18"/>
-      <c r="IG7" s="18"/>
-      <c r="IH7" s="18"/>
-      <c r="II7" s="18"/>
-      <c r="IJ7" s="18"/>
-      <c r="IK7" s="18"/>
-      <c r="IL7" s="18"/>
-      <c r="IM7" s="18"/>
-      <c r="IN7" s="18"/>
-      <c r="IO7" s="18"/>
-      <c r="IP7" s="18"/>
-      <c r="IQ7" s="18"/>
-      <c r="IR7" s="18"/>
-      <c r="IS7" s="18"/>
-      <c r="IT7" s="18"/>
-      <c r="IU7" s="18"/>
-      <c r="IV7" s="18"/>
-      <c r="IW7" s="18"/>
+      <c r="M7" s="45"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="15"/>
+      <c r="S7" s="15"/>
+      <c r="T7" s="15"/>
+      <c r="U7" s="15"/>
+      <c r="V7" s="15"/>
+      <c r="W7" s="15"/>
+      <c r="X7" s="15"/>
+      <c r="Y7" s="15"/>
+      <c r="Z7" s="15"/>
+      <c r="AA7" s="15"/>
+      <c r="AB7" s="15"/>
+      <c r="AC7" s="15"/>
+      <c r="AD7" s="15"/>
+      <c r="AE7" s="15"/>
+      <c r="AF7" s="15"/>
+      <c r="AG7" s="15"/>
+      <c r="AH7" s="15"/>
+      <c r="AI7" s="15"/>
+      <c r="AJ7" s="15"/>
+      <c r="AK7" s="15"/>
+      <c r="AL7" s="15"/>
+      <c r="AM7" s="15"/>
+      <c r="AN7" s="15"/>
+      <c r="AO7" s="15"/>
+      <c r="AP7" s="15"/>
+      <c r="AQ7" s="15"/>
+      <c r="AR7" s="15"/>
+      <c r="AS7" s="15"/>
+      <c r="AT7" s="15"/>
+      <c r="AU7" s="15"/>
+      <c r="AV7" s="15"/>
+      <c r="AW7" s="15"/>
+      <c r="AX7" s="15"/>
+      <c r="AY7" s="15"/>
+      <c r="AZ7" s="15"/>
+      <c r="BA7" s="15"/>
+      <c r="BB7" s="15"/>
+      <c r="BC7" s="15"/>
+      <c r="BD7" s="15"/>
+      <c r="BE7" s="15"/>
+      <c r="BF7" s="15"/>
+      <c r="BG7" s="15"/>
+      <c r="BH7" s="15"/>
+      <c r="BI7" s="15"/>
+      <c r="BJ7" s="15"/>
+      <c r="BK7" s="15"/>
+      <c r="BL7" s="15"/>
+      <c r="BM7" s="15"/>
+      <c r="BN7" s="15"/>
+      <c r="BO7" s="15"/>
+      <c r="BP7" s="15"/>
+      <c r="BQ7" s="15"/>
+      <c r="BR7" s="15"/>
+      <c r="BS7" s="15"/>
+      <c r="BT7" s="15"/>
+      <c r="BU7" s="15"/>
+      <c r="BV7" s="15"/>
+      <c r="BW7" s="15"/>
+      <c r="BX7" s="15"/>
+      <c r="BY7" s="15"/>
+      <c r="BZ7" s="15"/>
+      <c r="CA7" s="15"/>
+      <c r="CB7" s="15"/>
+      <c r="CC7" s="15"/>
+      <c r="CD7" s="15"/>
+      <c r="CE7" s="15"/>
+      <c r="CF7" s="15"/>
+      <c r="CG7" s="15"/>
+      <c r="CH7" s="15"/>
+      <c r="CI7" s="15"/>
+      <c r="CJ7" s="15"/>
+      <c r="CK7" s="15"/>
+      <c r="CL7" s="15"/>
+      <c r="CM7" s="15"/>
+      <c r="CN7" s="15"/>
+      <c r="CO7" s="15"/>
+      <c r="CP7" s="15"/>
+      <c r="CQ7" s="15"/>
+      <c r="CR7" s="15"/>
+      <c r="CS7" s="15"/>
+      <c r="CT7" s="15"/>
+      <c r="CU7" s="15"/>
+      <c r="CV7" s="15"/>
+      <c r="CW7" s="15"/>
+      <c r="CX7" s="15"/>
+      <c r="CY7" s="15"/>
+      <c r="CZ7" s="15"/>
+      <c r="DA7" s="15"/>
+      <c r="DB7" s="15"/>
+      <c r="DC7" s="15"/>
+      <c r="DD7" s="15"/>
+      <c r="DE7" s="15"/>
+      <c r="DF7" s="15"/>
+      <c r="DG7" s="15"/>
+      <c r="DH7" s="15"/>
+      <c r="DI7" s="15"/>
+      <c r="DJ7" s="15"/>
+      <c r="DK7" s="15"/>
+      <c r="DL7" s="15"/>
+      <c r="DM7" s="15"/>
+      <c r="DN7" s="15"/>
+      <c r="DO7" s="15"/>
+      <c r="DP7" s="15"/>
+      <c r="DQ7" s="15"/>
+      <c r="DR7" s="15"/>
+      <c r="DS7" s="15"/>
+      <c r="DT7" s="15"/>
+      <c r="DU7" s="15"/>
+      <c r="DV7" s="15"/>
+      <c r="DW7" s="15"/>
+      <c r="DX7" s="15"/>
+      <c r="DY7" s="15"/>
+      <c r="DZ7" s="15"/>
+      <c r="EA7" s="15"/>
+      <c r="EB7" s="15"/>
+      <c r="EC7" s="15"/>
+      <c r="ED7" s="15"/>
+      <c r="EE7" s="15"/>
+      <c r="EF7" s="15"/>
+      <c r="EG7" s="15"/>
+      <c r="EH7" s="15"/>
+      <c r="EI7" s="15"/>
+      <c r="EJ7" s="15"/>
+      <c r="EK7" s="15"/>
+      <c r="EL7" s="15"/>
+      <c r="EM7" s="15"/>
+      <c r="EN7" s="15"/>
+      <c r="EO7" s="15"/>
+      <c r="EP7" s="15"/>
+      <c r="EQ7" s="15"/>
+      <c r="ER7" s="15"/>
+      <c r="ES7" s="15"/>
+      <c r="ET7" s="15"/>
+      <c r="EU7" s="15"/>
+      <c r="EV7" s="15"/>
+      <c r="EW7" s="15"/>
+      <c r="EX7" s="15"/>
+      <c r="EY7" s="15"/>
+      <c r="EZ7" s="15"/>
+      <c r="FA7" s="15"/>
+      <c r="FB7" s="15"/>
+      <c r="FC7" s="15"/>
+      <c r="FD7" s="15"/>
+      <c r="FE7" s="15"/>
+      <c r="FF7" s="15"/>
+      <c r="FG7" s="15"/>
+      <c r="FH7" s="15"/>
+      <c r="FI7" s="15"/>
+      <c r="FJ7" s="15"/>
+      <c r="FK7" s="15"/>
+      <c r="FL7" s="15"/>
+      <c r="FM7" s="15"/>
+      <c r="FN7" s="15"/>
+      <c r="FO7" s="15"/>
+      <c r="FP7" s="15"/>
+      <c r="FQ7" s="15"/>
+      <c r="FR7" s="15"/>
+      <c r="FS7" s="15"/>
+      <c r="FT7" s="15"/>
+      <c r="FU7" s="15"/>
+      <c r="FV7" s="15"/>
+      <c r="FW7" s="15"/>
+      <c r="FX7" s="15"/>
+      <c r="FY7" s="15"/>
+      <c r="FZ7" s="15"/>
+      <c r="GA7" s="15"/>
+      <c r="GB7" s="15"/>
+      <c r="GC7" s="15"/>
+      <c r="GD7" s="15"/>
+      <c r="GE7" s="15"/>
+      <c r="GF7" s="15"/>
+      <c r="GG7" s="15"/>
+      <c r="GH7" s="15"/>
+      <c r="GI7" s="15"/>
+      <c r="GJ7" s="15"/>
+      <c r="GK7" s="15"/>
+      <c r="GL7" s="15"/>
+      <c r="GM7" s="15"/>
+      <c r="GN7" s="15"/>
+      <c r="GO7" s="15"/>
+      <c r="GP7" s="15"/>
+      <c r="GQ7" s="15"/>
+      <c r="GR7" s="15"/>
+      <c r="GS7" s="15"/>
+      <c r="GT7" s="15"/>
+      <c r="GU7" s="15"/>
+      <c r="GV7" s="15"/>
+      <c r="GW7" s="15"/>
+      <c r="GX7" s="15"/>
+      <c r="GY7" s="15"/>
+      <c r="GZ7" s="15"/>
+      <c r="HA7" s="15"/>
+      <c r="HB7" s="15"/>
+      <c r="HC7" s="15"/>
+      <c r="HD7" s="15"/>
+      <c r="HE7" s="15"/>
+      <c r="HF7" s="15"/>
+      <c r="HG7" s="15"/>
+      <c r="HH7" s="15"/>
+      <c r="HI7" s="15"/>
+      <c r="HJ7" s="15"/>
+      <c r="HK7" s="15"/>
+      <c r="HL7" s="15"/>
+      <c r="HM7" s="15"/>
+      <c r="HN7" s="15"/>
+      <c r="HO7" s="15"/>
+      <c r="HP7" s="15"/>
+      <c r="HQ7" s="15"/>
+      <c r="HR7" s="15"/>
+      <c r="HS7" s="15"/>
+      <c r="HT7" s="15"/>
+      <c r="HU7" s="15"/>
+      <c r="HV7" s="15"/>
+      <c r="HW7" s="15"/>
+      <c r="HX7" s="15"/>
+      <c r="HY7" s="15"/>
+      <c r="HZ7" s="15"/>
+      <c r="IA7" s="15"/>
+      <c r="IB7" s="15"/>
+      <c r="IC7" s="15"/>
+      <c r="ID7" s="15"/>
+      <c r="IE7" s="15"/>
+      <c r="IF7" s="15"/>
+      <c r="IG7" s="15"/>
+      <c r="IH7" s="15"/>
+      <c r="II7" s="15"/>
+      <c r="IJ7" s="15"/>
+      <c r="IK7" s="15"/>
+      <c r="IL7" s="15"/>
+      <c r="IM7" s="15"/>
+      <c r="IN7" s="15"/>
+      <c r="IO7" s="15"/>
+      <c r="IP7" s="15"/>
+      <c r="IQ7" s="15"/>
+      <c r="IR7" s="15"/>
+      <c r="IS7" s="15"/>
+      <c r="IT7" s="15"/>
+      <c r="IU7" s="15"/>
+      <c r="IV7" s="15"/>
+      <c r="IW7" s="15"/>
     </row>
     <row r="8" spans="1:257" ht="18" customHeight="1">
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+      <c r="G8" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="10" spans="1:257" ht="17.399999999999999">
       <c r="A10" s="3">
         <f>D2</f>
-        <v>-134.98539803417327</v>
+        <v>-1.32</v>
       </c>
       <c r="B10" s="3">
         <f>E2</f>
-        <v>160.86933305498539</v>
+        <v>1.58</v>
       </c>
       <c r="C10" s="3">
         <f>D3</f>
-        <v>234.92315519647701</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="D10" s="3">
         <f>E3</f>
-        <v>-85.505035831417359</v>
+        <v>-0.84</v>
       </c>
       <c r="E10" s="3">
         <f>D4</f>
-        <v>-99.93775716230374</v>
+        <v>-0.98</v>
       </c>
       <c r="F10" s="3">
         <f>E4</f>
-        <v>-75.36429722356803</v>
+        <v>-0.74</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
@@ -3604,12 +3840,12 @@
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="47"/>
+      <c r="K11" s="47"/>
+      <c r="L11" s="47"/>
+      <c r="M11" s="47"/>
+      <c r="N11" s="47"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
@@ -3855,128 +4091,74 @@
       <c r="IW11" s="3"/>
     </row>
     <row r="12" spans="1:257" ht="18" customHeight="1">
-      <c r="I12" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="L12" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="M12" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="G12" s="33">
+        <v>20</v>
+      </c>
+      <c r="I12" s="48"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="50"/>
+      <c r="L12" s="48"/>
+      <c r="M12" s="48"/>
+      <c r="N12" s="36"/>
     </row>
     <row r="13" spans="1:257" ht="18" customHeight="1">
-      <c r="I13" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J13" s="9">
-        <v>150</v>
-      </c>
-      <c r="K13" s="9">
-        <v>130</v>
-      </c>
-      <c r="L13" s="10">
-        <f>J13*COS(K13/180*PI())</f>
-        <v>-96.418141452980905</v>
-      </c>
-      <c r="M13" s="10">
-        <f>J13*SIN(K13/180*PI())</f>
-        <v>114.9066664678467</v>
-      </c>
+      <c r="G13" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" s="51"/>
+      <c r="J13" s="60"/>
+      <c r="K13" s="60"/>
+      <c r="L13" s="52"/>
+      <c r="M13" s="52"/>
+      <c r="N13" s="36"/>
     </row>
     <row r="14" spans="1:257" ht="18" customHeight="1">
-      <c r="I14" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="J14" s="9">
-        <v>200</v>
-      </c>
-      <c r="K14" s="9">
-        <v>90</v>
-      </c>
-      <c r="L14" s="10">
-        <f>J14*COS(K14/180*PI())</f>
-        <v>1.22514845490862E-14</v>
-      </c>
-      <c r="M14" s="10">
-        <f>J14*SIN(K14/180*PI())</f>
-        <v>200</v>
-      </c>
+      <c r="I14" s="51"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="60"/>
+      <c r="L14" s="52"/>
+      <c r="M14" s="52"/>
+      <c r="N14" s="36"/>
     </row>
     <row r="15" spans="1:257" ht="18" customHeight="1">
-      <c r="I15" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J15" s="12">
-        <f>(L15^2+M15^2)^0.5</f>
-        <v>329.33670701447585</v>
-      </c>
-      <c r="K15" s="12">
-        <f>IF(L15&lt;0,(IF(M15&lt;0,ATAN(M15/L15)*(180/PI())+180,ATAN(M15/L15)*(180/PI())+180)),(IF(M15&lt;0,ATAN(M15/L15)*(180/PI())+360,ATAN(M15/L15)*(180/PI()))))</f>
-        <v>287.02354351077287</v>
-      </c>
-      <c r="L15" s="12">
-        <f>-L13-L14</f>
-        <v>96.41814145298089</v>
-      </c>
-      <c r="M15" s="12">
-        <f>-M13-M14</f>
-        <v>-314.90666646784672</v>
-      </c>
+      <c r="I15" s="51"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="61"/>
+      <c r="L15" s="53"/>
+      <c r="M15" s="53"/>
+      <c r="N15" s="36"/>
     </row>
     <row r="16" spans="1:257" ht="18" customHeight="1">
-      <c r="I16" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="J16" s="13">
-        <v>250</v>
-      </c>
-      <c r="K16" s="9">
-        <v>233.13</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="M16" s="14"/>
+      <c r="I16" s="51"/>
+      <c r="J16" s="62"/>
+      <c r="K16" s="60"/>
+      <c r="L16" s="54"/>
+      <c r="M16" s="54"/>
+      <c r="N16" s="36"/>
     </row>
-    <row r="17" spans="8:13" ht="18" customHeight="1">
-      <c r="I17" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J17" s="12">
-        <f>J15-J16</f>
-        <v>79.336707014475849</v>
-      </c>
-      <c r="K17" s="12">
-        <f>K15-K16</f>
-        <v>53.893543510772872</v>
-      </c>
-      <c r="L17" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="M17" s="14"/>
+    <row r="17" spans="8:14" ht="18" customHeight="1">
+      <c r="H17" s="58"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="53"/>
+      <c r="K17" s="53"/>
+      <c r="L17" s="54"/>
+      <c r="M17" s="54"/>
+      <c r="N17" s="36"/>
     </row>
-    <row r="18" spans="8:13" ht="18" customHeight="1">
-      <c r="I18" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J18" s="15">
-        <f>ABS((J16-J15)/((J16+J15)/2))*100</f>
-        <v>27.3888072528066</v>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="M18" s="17"/>
+    <row r="18" spans="8:14" ht="18" customHeight="1">
+      <c r="H18" s="58"/>
+      <c r="I18" s="59"/>
+      <c r="J18" s="55"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="57"/>
+      <c r="M18" s="57"/>
+      <c r="N18" s="36"/>
     </row>
-    <row r="22" spans="8:13" ht="18" customHeight="1">
+    <row r="19" spans="8:14" ht="18" customHeight="1">
+      <c r="H19" s="58"/>
+      <c r="I19" s="58"/>
+    </row>
+    <row r="22" spans="8:14" ht="18" customHeight="1">
       <c r="I22" s="4" t="s">
         <v>1</v>
       </c>
@@ -3984,13 +4166,13 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="8:13" ht="18" customHeight="1">
+    <row r="23" spans="8:14" ht="18" customHeight="1">
       <c r="H23"/>
       <c r="I23"/>
       <c r="J23"/>
     </row>
     <row r="37" spans="1:257" ht="17.399999999999999">
-      <c r="A37" s="19">
+      <c r="A37" s="16">
         <v>4</v>
       </c>
     </row>
@@ -4010,258 +4192,258 @@
       <c r="E38" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F38" s="20"/>
-      <c r="G38" s="20"/>
-      <c r="H38" s="20"/>
-      <c r="I38" s="20"/>
-      <c r="J38" s="20"/>
-      <c r="K38" s="20"/>
-      <c r="L38" s="20"/>
-      <c r="M38" s="20"/>
-      <c r="N38" s="20"/>
-      <c r="O38" s="20"/>
-      <c r="P38" s="20"/>
-      <c r="Q38" s="20"/>
-      <c r="R38" s="20"/>
-      <c r="S38" s="20"/>
-      <c r="T38" s="20"/>
-      <c r="U38" s="20"/>
-      <c r="V38" s="20"/>
-      <c r="W38" s="20"/>
-      <c r="X38" s="20"/>
-      <c r="Y38" s="20"/>
-      <c r="Z38" s="20"/>
-      <c r="AA38" s="20"/>
-      <c r="AB38" s="20"/>
-      <c r="AC38" s="20"/>
-      <c r="AD38" s="20"/>
-      <c r="AE38" s="20"/>
-      <c r="AF38" s="20"/>
-      <c r="AG38" s="20"/>
-      <c r="AH38" s="20"/>
-      <c r="AI38" s="20"/>
-      <c r="AJ38" s="20"/>
-      <c r="AK38" s="20"/>
-      <c r="AL38" s="20"/>
-      <c r="AM38" s="20"/>
-      <c r="AN38" s="20"/>
-      <c r="AO38" s="20"/>
-      <c r="AP38" s="20"/>
-      <c r="AQ38" s="20"/>
-      <c r="AR38" s="20"/>
-      <c r="AS38" s="20"/>
-      <c r="AT38" s="20"/>
-      <c r="AU38" s="20"/>
-      <c r="AV38" s="20"/>
-      <c r="AW38" s="20"/>
-      <c r="AX38" s="20"/>
-      <c r="AY38" s="20"/>
-      <c r="AZ38" s="20"/>
-      <c r="BA38" s="20"/>
-      <c r="BB38" s="20"/>
-      <c r="BC38" s="20"/>
-      <c r="BD38" s="20"/>
-      <c r="BE38" s="20"/>
-      <c r="BF38" s="20"/>
-      <c r="BG38" s="20"/>
-      <c r="BH38" s="20"/>
-      <c r="BI38" s="20"/>
-      <c r="BJ38" s="20"/>
-      <c r="BK38" s="20"/>
-      <c r="BL38" s="20"/>
-      <c r="BM38" s="20"/>
-      <c r="BN38" s="20"/>
-      <c r="BO38" s="20"/>
-      <c r="BP38" s="20"/>
-      <c r="BQ38" s="20"/>
-      <c r="BR38" s="20"/>
-      <c r="BS38" s="20"/>
-      <c r="BT38" s="20"/>
-      <c r="BU38" s="20"/>
-      <c r="BV38" s="20"/>
-      <c r="BW38" s="20"/>
-      <c r="BX38" s="20"/>
-      <c r="BY38" s="20"/>
-      <c r="BZ38" s="20"/>
-      <c r="CA38" s="20"/>
-      <c r="CB38" s="20"/>
-      <c r="CC38" s="20"/>
-      <c r="CD38" s="20"/>
-      <c r="CE38" s="20"/>
-      <c r="CF38" s="20"/>
-      <c r="CG38" s="20"/>
-      <c r="CH38" s="20"/>
-      <c r="CI38" s="20"/>
-      <c r="CJ38" s="20"/>
-      <c r="CK38" s="20"/>
-      <c r="CL38" s="20"/>
-      <c r="CM38" s="20"/>
-      <c r="CN38" s="20"/>
-      <c r="CO38" s="20"/>
-      <c r="CP38" s="20"/>
-      <c r="CQ38" s="20"/>
-      <c r="CR38" s="20"/>
-      <c r="CS38" s="20"/>
-      <c r="CT38" s="20"/>
-      <c r="CU38" s="20"/>
-      <c r="CV38" s="20"/>
-      <c r="CW38" s="20"/>
-      <c r="CX38" s="20"/>
-      <c r="CY38" s="20"/>
-      <c r="CZ38" s="20"/>
-      <c r="DA38" s="20"/>
-      <c r="DB38" s="20"/>
-      <c r="DC38" s="20"/>
-      <c r="DD38" s="20"/>
-      <c r="DE38" s="20"/>
-      <c r="DF38" s="20"/>
-      <c r="DG38" s="20"/>
-      <c r="DH38" s="20"/>
-      <c r="DI38" s="20"/>
-      <c r="DJ38" s="20"/>
-      <c r="DK38" s="20"/>
-      <c r="DL38" s="20"/>
-      <c r="DM38" s="20"/>
-      <c r="DN38" s="20"/>
-      <c r="DO38" s="20"/>
-      <c r="DP38" s="20"/>
-      <c r="DQ38" s="20"/>
-      <c r="DR38" s="20"/>
-      <c r="DS38" s="20"/>
-      <c r="DT38" s="20"/>
-      <c r="DU38" s="20"/>
-      <c r="DV38" s="20"/>
-      <c r="DW38" s="20"/>
-      <c r="DX38" s="20"/>
-      <c r="DY38" s="20"/>
-      <c r="DZ38" s="20"/>
-      <c r="EA38" s="20"/>
-      <c r="EB38" s="20"/>
-      <c r="EC38" s="20"/>
-      <c r="ED38" s="20"/>
-      <c r="EE38" s="20"/>
-      <c r="EF38" s="20"/>
-      <c r="EG38" s="20"/>
-      <c r="EH38" s="20"/>
-      <c r="EI38" s="20"/>
-      <c r="EJ38" s="20"/>
-      <c r="EK38" s="20"/>
-      <c r="EL38" s="20"/>
-      <c r="EM38" s="20"/>
-      <c r="EN38" s="20"/>
-      <c r="EO38" s="20"/>
-      <c r="EP38" s="20"/>
-      <c r="EQ38" s="20"/>
-      <c r="ER38" s="20"/>
-      <c r="ES38" s="20"/>
-      <c r="ET38" s="20"/>
-      <c r="EU38" s="20"/>
-      <c r="EV38" s="20"/>
-      <c r="EW38" s="20"/>
-      <c r="EX38" s="20"/>
-      <c r="EY38" s="20"/>
-      <c r="EZ38" s="20"/>
-      <c r="FA38" s="20"/>
-      <c r="FB38" s="20"/>
-      <c r="FC38" s="20"/>
-      <c r="FD38" s="20"/>
-      <c r="FE38" s="20"/>
-      <c r="FF38" s="20"/>
-      <c r="FG38" s="20"/>
-      <c r="FH38" s="20"/>
-      <c r="FI38" s="20"/>
-      <c r="FJ38" s="20"/>
-      <c r="FK38" s="20"/>
-      <c r="FL38" s="20"/>
-      <c r="FM38" s="20"/>
-      <c r="FN38" s="20"/>
-      <c r="FO38" s="20"/>
-      <c r="FP38" s="20"/>
-      <c r="FQ38" s="20"/>
-      <c r="FR38" s="20"/>
-      <c r="FS38" s="20"/>
-      <c r="FT38" s="20"/>
-      <c r="FU38" s="20"/>
-      <c r="FV38" s="20"/>
-      <c r="FW38" s="20"/>
-      <c r="FX38" s="20"/>
-      <c r="FY38" s="20"/>
-      <c r="FZ38" s="20"/>
-      <c r="GA38" s="20"/>
-      <c r="GB38" s="20"/>
-      <c r="GC38" s="20"/>
-      <c r="GD38" s="20"/>
-      <c r="GE38" s="20"/>
-      <c r="GF38" s="20"/>
-      <c r="GG38" s="20"/>
-      <c r="GH38" s="20"/>
-      <c r="GI38" s="20"/>
-      <c r="GJ38" s="20"/>
-      <c r="GK38" s="20"/>
-      <c r="GL38" s="20"/>
-      <c r="GM38" s="20"/>
-      <c r="GN38" s="20"/>
-      <c r="GO38" s="20"/>
-      <c r="GP38" s="20"/>
-      <c r="GQ38" s="20"/>
-      <c r="GR38" s="20"/>
-      <c r="GS38" s="20"/>
-      <c r="GT38" s="20"/>
-      <c r="GU38" s="20"/>
-      <c r="GV38" s="20"/>
-      <c r="GW38" s="20"/>
-      <c r="GX38" s="20"/>
-      <c r="GY38" s="20"/>
-      <c r="GZ38" s="20"/>
-      <c r="HA38" s="20"/>
-      <c r="HB38" s="20"/>
-      <c r="HC38" s="20"/>
-      <c r="HD38" s="20"/>
-      <c r="HE38" s="20"/>
-      <c r="HF38" s="20"/>
-      <c r="HG38" s="20"/>
-      <c r="HH38" s="20"/>
-      <c r="HI38" s="20"/>
-      <c r="HJ38" s="20"/>
-      <c r="HK38" s="20"/>
-      <c r="HL38" s="20"/>
-      <c r="HM38" s="20"/>
-      <c r="HN38" s="20"/>
-      <c r="HO38" s="20"/>
-      <c r="HP38" s="20"/>
-      <c r="HQ38" s="20"/>
-      <c r="HR38" s="20"/>
-      <c r="HS38" s="20"/>
-      <c r="HT38" s="20"/>
-      <c r="HU38" s="20"/>
-      <c r="HV38" s="20"/>
-      <c r="HW38" s="20"/>
-      <c r="HX38" s="20"/>
-      <c r="HY38" s="20"/>
-      <c r="HZ38" s="20"/>
-      <c r="IA38" s="20"/>
-      <c r="IB38" s="20"/>
-      <c r="IC38" s="20"/>
-      <c r="ID38" s="20"/>
-      <c r="IE38" s="20"/>
-      <c r="IF38" s="20"/>
-      <c r="IG38" s="20"/>
-      <c r="IH38" s="20"/>
-      <c r="II38" s="20"/>
-      <c r="IJ38" s="20"/>
-      <c r="IK38" s="20"/>
-      <c r="IL38" s="20"/>
-      <c r="IM38" s="20"/>
-      <c r="IN38" s="20"/>
-      <c r="IO38" s="20"/>
-      <c r="IP38" s="20"/>
-      <c r="IQ38" s="20"/>
-      <c r="IR38" s="20"/>
-      <c r="IS38" s="20"/>
-      <c r="IT38" s="20"/>
-      <c r="IU38" s="20"/>
-      <c r="IV38" s="20"/>
-      <c r="IW38" s="20"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
+      <c r="N38" s="17"/>
+      <c r="O38" s="17"/>
+      <c r="P38" s="17"/>
+      <c r="Q38" s="17"/>
+      <c r="R38" s="17"/>
+      <c r="S38" s="17"/>
+      <c r="T38" s="17"/>
+      <c r="U38" s="17"/>
+      <c r="V38" s="17"/>
+      <c r="W38" s="17"/>
+      <c r="X38" s="17"/>
+      <c r="Y38" s="17"/>
+      <c r="Z38" s="17"/>
+      <c r="AA38" s="17"/>
+      <c r="AB38" s="17"/>
+      <c r="AC38" s="17"/>
+      <c r="AD38" s="17"/>
+      <c r="AE38" s="17"/>
+      <c r="AF38" s="17"/>
+      <c r="AG38" s="17"/>
+      <c r="AH38" s="17"/>
+      <c r="AI38" s="17"/>
+      <c r="AJ38" s="17"/>
+      <c r="AK38" s="17"/>
+      <c r="AL38" s="17"/>
+      <c r="AM38" s="17"/>
+      <c r="AN38" s="17"/>
+      <c r="AO38" s="17"/>
+      <c r="AP38" s="17"/>
+      <c r="AQ38" s="17"/>
+      <c r="AR38" s="17"/>
+      <c r="AS38" s="17"/>
+      <c r="AT38" s="17"/>
+      <c r="AU38" s="17"/>
+      <c r="AV38" s="17"/>
+      <c r="AW38" s="17"/>
+      <c r="AX38" s="17"/>
+      <c r="AY38" s="17"/>
+      <c r="AZ38" s="17"/>
+      <c r="BA38" s="17"/>
+      <c r="BB38" s="17"/>
+      <c r="BC38" s="17"/>
+      <c r="BD38" s="17"/>
+      <c r="BE38" s="17"/>
+      <c r="BF38" s="17"/>
+      <c r="BG38" s="17"/>
+      <c r="BH38" s="17"/>
+      <c r="BI38" s="17"/>
+      <c r="BJ38" s="17"/>
+      <c r="BK38" s="17"/>
+      <c r="BL38" s="17"/>
+      <c r="BM38" s="17"/>
+      <c r="BN38" s="17"/>
+      <c r="BO38" s="17"/>
+      <c r="BP38" s="17"/>
+      <c r="BQ38" s="17"/>
+      <c r="BR38" s="17"/>
+      <c r="BS38" s="17"/>
+      <c r="BT38" s="17"/>
+      <c r="BU38" s="17"/>
+      <c r="BV38" s="17"/>
+      <c r="BW38" s="17"/>
+      <c r="BX38" s="17"/>
+      <c r="BY38" s="17"/>
+      <c r="BZ38" s="17"/>
+      <c r="CA38" s="17"/>
+      <c r="CB38" s="17"/>
+      <c r="CC38" s="17"/>
+      <c r="CD38" s="17"/>
+      <c r="CE38" s="17"/>
+      <c r="CF38" s="17"/>
+      <c r="CG38" s="17"/>
+      <c r="CH38" s="17"/>
+      <c r="CI38" s="17"/>
+      <c r="CJ38" s="17"/>
+      <c r="CK38" s="17"/>
+      <c r="CL38" s="17"/>
+      <c r="CM38" s="17"/>
+      <c r="CN38" s="17"/>
+      <c r="CO38" s="17"/>
+      <c r="CP38" s="17"/>
+      <c r="CQ38" s="17"/>
+      <c r="CR38" s="17"/>
+      <c r="CS38" s="17"/>
+      <c r="CT38" s="17"/>
+      <c r="CU38" s="17"/>
+      <c r="CV38" s="17"/>
+      <c r="CW38" s="17"/>
+      <c r="CX38" s="17"/>
+      <c r="CY38" s="17"/>
+      <c r="CZ38" s="17"/>
+      <c r="DA38" s="17"/>
+      <c r="DB38" s="17"/>
+      <c r="DC38" s="17"/>
+      <c r="DD38" s="17"/>
+      <c r="DE38" s="17"/>
+      <c r="DF38" s="17"/>
+      <c r="DG38" s="17"/>
+      <c r="DH38" s="17"/>
+      <c r="DI38" s="17"/>
+      <c r="DJ38" s="17"/>
+      <c r="DK38" s="17"/>
+      <c r="DL38" s="17"/>
+      <c r="DM38" s="17"/>
+      <c r="DN38" s="17"/>
+      <c r="DO38" s="17"/>
+      <c r="DP38" s="17"/>
+      <c r="DQ38" s="17"/>
+      <c r="DR38" s="17"/>
+      <c r="DS38" s="17"/>
+      <c r="DT38" s="17"/>
+      <c r="DU38" s="17"/>
+      <c r="DV38" s="17"/>
+      <c r="DW38" s="17"/>
+      <c r="DX38" s="17"/>
+      <c r="DY38" s="17"/>
+      <c r="DZ38" s="17"/>
+      <c r="EA38" s="17"/>
+      <c r="EB38" s="17"/>
+      <c r="EC38" s="17"/>
+      <c r="ED38" s="17"/>
+      <c r="EE38" s="17"/>
+      <c r="EF38" s="17"/>
+      <c r="EG38" s="17"/>
+      <c r="EH38" s="17"/>
+      <c r="EI38" s="17"/>
+      <c r="EJ38" s="17"/>
+      <c r="EK38" s="17"/>
+      <c r="EL38" s="17"/>
+      <c r="EM38" s="17"/>
+      <c r="EN38" s="17"/>
+      <c r="EO38" s="17"/>
+      <c r="EP38" s="17"/>
+      <c r="EQ38" s="17"/>
+      <c r="ER38" s="17"/>
+      <c r="ES38" s="17"/>
+      <c r="ET38" s="17"/>
+      <c r="EU38" s="17"/>
+      <c r="EV38" s="17"/>
+      <c r="EW38" s="17"/>
+      <c r="EX38" s="17"/>
+      <c r="EY38" s="17"/>
+      <c r="EZ38" s="17"/>
+      <c r="FA38" s="17"/>
+      <c r="FB38" s="17"/>
+      <c r="FC38" s="17"/>
+      <c r="FD38" s="17"/>
+      <c r="FE38" s="17"/>
+      <c r="FF38" s="17"/>
+      <c r="FG38" s="17"/>
+      <c r="FH38" s="17"/>
+      <c r="FI38" s="17"/>
+      <c r="FJ38" s="17"/>
+      <c r="FK38" s="17"/>
+      <c r="FL38" s="17"/>
+      <c r="FM38" s="17"/>
+      <c r="FN38" s="17"/>
+      <c r="FO38" s="17"/>
+      <c r="FP38" s="17"/>
+      <c r="FQ38" s="17"/>
+      <c r="FR38" s="17"/>
+      <c r="FS38" s="17"/>
+      <c r="FT38" s="17"/>
+      <c r="FU38" s="17"/>
+      <c r="FV38" s="17"/>
+      <c r="FW38" s="17"/>
+      <c r="FX38" s="17"/>
+      <c r="FY38" s="17"/>
+      <c r="FZ38" s="17"/>
+      <c r="GA38" s="17"/>
+      <c r="GB38" s="17"/>
+      <c r="GC38" s="17"/>
+      <c r="GD38" s="17"/>
+      <c r="GE38" s="17"/>
+      <c r="GF38" s="17"/>
+      <c r="GG38" s="17"/>
+      <c r="GH38" s="17"/>
+      <c r="GI38" s="17"/>
+      <c r="GJ38" s="17"/>
+      <c r="GK38" s="17"/>
+      <c r="GL38" s="17"/>
+      <c r="GM38" s="17"/>
+      <c r="GN38" s="17"/>
+      <c r="GO38" s="17"/>
+      <c r="GP38" s="17"/>
+      <c r="GQ38" s="17"/>
+      <c r="GR38" s="17"/>
+      <c r="GS38" s="17"/>
+      <c r="GT38" s="17"/>
+      <c r="GU38" s="17"/>
+      <c r="GV38" s="17"/>
+      <c r="GW38" s="17"/>
+      <c r="GX38" s="17"/>
+      <c r="GY38" s="17"/>
+      <c r="GZ38" s="17"/>
+      <c r="HA38" s="17"/>
+      <c r="HB38" s="17"/>
+      <c r="HC38" s="17"/>
+      <c r="HD38" s="17"/>
+      <c r="HE38" s="17"/>
+      <c r="HF38" s="17"/>
+      <c r="HG38" s="17"/>
+      <c r="HH38" s="17"/>
+      <c r="HI38" s="17"/>
+      <c r="HJ38" s="17"/>
+      <c r="HK38" s="17"/>
+      <c r="HL38" s="17"/>
+      <c r="HM38" s="17"/>
+      <c r="HN38" s="17"/>
+      <c r="HO38" s="17"/>
+      <c r="HP38" s="17"/>
+      <c r="HQ38" s="17"/>
+      <c r="HR38" s="17"/>
+      <c r="HS38" s="17"/>
+      <c r="HT38" s="17"/>
+      <c r="HU38" s="17"/>
+      <c r="HV38" s="17"/>
+      <c r="HW38" s="17"/>
+      <c r="HX38" s="17"/>
+      <c r="HY38" s="17"/>
+      <c r="HZ38" s="17"/>
+      <c r="IA38" s="17"/>
+      <c r="IB38" s="17"/>
+      <c r="IC38" s="17"/>
+      <c r="ID38" s="17"/>
+      <c r="IE38" s="17"/>
+      <c r="IF38" s="17"/>
+      <c r="IG38" s="17"/>
+      <c r="IH38" s="17"/>
+      <c r="II38" s="17"/>
+      <c r="IJ38" s="17"/>
+      <c r="IK38" s="17"/>
+      <c r="IL38" s="17"/>
+      <c r="IM38" s="17"/>
+      <c r="IN38" s="17"/>
+      <c r="IO38" s="17"/>
+      <c r="IP38" s="17"/>
+      <c r="IQ38" s="17"/>
+      <c r="IR38" s="17"/>
+      <c r="IS38" s="17"/>
+      <c r="IT38" s="17"/>
+      <c r="IU38" s="17"/>
+      <c r="IV38" s="17"/>
+      <c r="IW38" s="17"/>
     </row>
     <row r="39" spans="1:257" ht="17.399999999999999">
       <c r="A39" s="8" t="s">
@@ -4273,11 +4455,11 @@
       <c r="C39" s="9">
         <v>130</v>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="18">
         <f>B39*COS(C39/180*PI())</f>
         <v>-134.98539803417327</v>
       </c>
-      <c r="E39" s="21">
+      <c r="E39" s="18">
         <f>B39*SIN(C39/180*PI())</f>
         <v>160.86933305498539</v>
       </c>
@@ -4292,11 +4474,11 @@
       <c r="C40" s="9">
         <v>340</v>
       </c>
-      <c r="D40" s="21">
+      <c r="D40" s="18">
         <f>B40*COS(C40/180*PI())</f>
         <v>234.92315519647701</v>
       </c>
-      <c r="E40" s="21">
+      <c r="E40" s="18">
         <f>B40*SIN(C40/180*PI())</f>
         <v>-85.505035831417359</v>
       </c>
@@ -4308,19 +4490,19 @@
       <c r="A41" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B41" s="12">
+      <c r="B41" s="11">
         <f>(D41^2+E41^2)^0.5</f>
         <v>125.16921587448687</v>
       </c>
-      <c r="C41" s="12">
+      <c r="C41" s="11">
         <f>IF(D41&lt;0,(IF(E41&lt;0,ATAN(E41/D41)*57.693+180,ATAN(E41/D41)*57.693+180)),(IF(E41&lt;0,ATAN(E41/D41)*57.693+360,ATAN(E41/D41)*57.693)))</f>
         <v>217.2770525393401</v>
       </c>
-      <c r="D41" s="15">
+      <c r="D41" s="13">
         <f>-D39-D40</f>
         <v>-99.93775716230374</v>
       </c>
-      <c r="E41" s="15">
+      <c r="E41" s="13">
         <f>-E39-E40</f>
         <v>-75.36429722356803</v>
       </c>
@@ -4332,47 +4514,47 @@
       <c r="A42" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B42" s="13">
+      <c r="B42" s="12">
         <v>122</v>
       </c>
       <c r="C42" s="9">
         <v>215</v>
       </c>
-      <c r="D42" s="17" t="s">
+      <c r="D42" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E42" s="17"/>
+      <c r="E42" s="14"/>
     </row>
     <row r="43" spans="1:257" ht="17.399999999999999">
       <c r="A43" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B43" s="12">
+      <c r="B43" s="11">
         <f>B41-B42</f>
         <v>3.1692158744868664</v>
       </c>
-      <c r="C43" s="12">
+      <c r="C43" s="11">
         <f>C41-C42</f>
         <v>2.2770525393401044</v>
       </c>
-      <c r="D43" s="17" t="s">
+      <c r="D43" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E43" s="17"/>
+      <c r="E43" s="14"/>
     </row>
     <row r="44" spans="1:257" ht="17.399999999999999">
       <c r="A44" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B44" s="12">
+      <c r="B44" s="11">
         <f>ABS((B42-B41)/((B42+B41)/2))*100</f>
         <v>2.5644098625099025</v>
       </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="17" t="s">
+      <c r="C44" s="19"/>
+      <c r="D44" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E44" s="17"/>
+      <c r="E44" s="14"/>
     </row>
   </sheetData>
   <printOptions headings="1" gridLines="1"/>
@@ -4395,26 +4577,26 @@
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.109375" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" style="23" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" style="20" customWidth="1"/>
     <col min="3" max="3" width="89.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" style="23" customWidth="1"/>
-    <col min="5" max="5" width="15.44140625" style="23" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" style="20" customWidth="1"/>
+    <col min="5" max="5" width="15.44140625" style="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="23" t="s">
         <v>4</v>
       </c>
     </row>
@@ -4422,17 +4604,17 @@
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="27">
+      <c r="B2" s="24">
         <v>2.94</v>
       </c>
-      <c r="C2" s="28">
+      <c r="C2" s="25">
         <v>300</v>
       </c>
-      <c r="D2" s="24">
+      <c r="D2" s="21">
         <f>B2*COS(C2/180*3.1416)</f>
         <v>1.4700311745613521</v>
       </c>
-      <c r="E2" s="24">
+      <c r="E2" s="21">
         <f>B2*SIN(C2/180*3.1416)</f>
         <v>-2.5460966882303921</v>
       </c>
@@ -4441,17 +4623,17 @@
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="27">
+      <c r="B3" s="24">
         <v>3.92</v>
       </c>
-      <c r="C3" s="28">
+      <c r="C3" s="25">
         <v>320</v>
       </c>
-      <c r="D3" s="24">
+      <c r="D3" s="21">
         <f>B3*COS(C3/180*3.1416)</f>
         <v>3.0029271251281724</v>
       </c>
-      <c r="E3" s="24">
+      <c r="E3" s="21">
         <f>B3*SIN(C3/180*3.1416)</f>
         <v>-2.519688211102606</v>
       </c>
@@ -4460,19 +4642,19 @@
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="26">
         <f>(D4^2+E4^2)^0.5</f>
         <v>6.7579236897934587</v>
       </c>
-      <c r="C4" s="30">
+      <c r="C4" s="27">
         <f>IF(D4&lt;0,(IF(E4&lt;0,ATAN(E4/D4)*57.693+180,ATAN(E4/D4)*57.693+180)),(IF(E4&lt;0,ATAN(E4/D4)*57.693+360,ATAN(E4/D4)*57.693)))</f>
         <v>131.1070476696222</v>
       </c>
-      <c r="D4" s="29">
+      <c r="D4" s="26">
         <f>-D2-D3</f>
         <v>-4.472958299689525</v>
       </c>
-      <c r="E4" s="29">
+      <c r="E4" s="26">
         <f>-E2-E3</f>
         <v>5.0657848993329981</v>
       </c>
@@ -4481,13 +4663,13 @@
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="31">
+      <c r="B5" s="28">
         <v>4.8</v>
       </c>
-      <c r="C5" s="32">
+      <c r="C5" s="29">
         <v>131</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="20" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4495,15 +4677,15 @@
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="26">
         <f>B4-B5</f>
         <v>1.9579236897934589</v>
       </c>
-      <c r="C6" s="33">
+      <c r="C6" s="30">
         <f>C4-C5</f>
         <v>0.10704766962220447</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="20" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4511,14 +4693,14 @@
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="29">
+      <c r="B7" s="26">
         <f>ABS((B5-B4)/((B5+B4)/2))*100</f>
         <v>33.880197556979155</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="20" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>